<commit_message>
update inject mutasi sewing to contain packing section too
</commit_message>
<xml_diff>
--- a/public/assets/example/contoh-import-inject-mutasi-sewing.xlsx
+++ b/public/assets/example/contoh-import-inject-mutasi-sewing.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASBAZAR\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\nds_wip_local_main\public\assets\example\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{602EA3C6-EF05-4BF1-969C-3416DA2E793D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09323E26-BE90-4A2A-92DF-5FBB925603B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
   <si>
     <t>tgl_saldo</t>
   </si>
@@ -163,13 +163,19 @@
   </si>
   <si>
     <t>SEWING</t>
+  </si>
+  <si>
+    <t>pc_terima</t>
+  </si>
+  <si>
+    <t>pc_packing_scan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -223,9 +229,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -263,7 +269,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -369,7 +375,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -511,7 +517,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -519,8 +525,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AN7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -560,7 +566,7 @@
     <col min="38" max="38" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:40">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -675,8 +681,14 @@
       <c r="AL1" t="s">
         <v>37</v>
       </c>
+      <c r="AM1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>46</v>
+      </c>
     </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:40">
       <c r="A2" s="1">
         <v>46170</v>
       </c>
@@ -699,7 +711,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:40">
       <c r="A3" s="1">
         <v>46170</v>
       </c>
@@ -722,13 +734,13 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:40">
       <c r="A5" s="1"/>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:40">
       <c r="A6" s="1"/>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:40">
       <c r="A7" s="1"/>
     </row>
   </sheetData>

</xml_diff>